<commit_message>
#4 JLCPCB BOM update
</commit_message>
<xml_diff>
--- a/Design-Files/Main-Board-V1.0.0/Deliverables/BOM/Client-BOM-Main-Board-V1.0.0.xlsx
+++ b/Design-Files/Main-Board-V1.0.0/Deliverables/BOM/Client-BOM-Main-Board-V1.0.0.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="420" uniqueCount="275">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="413" uniqueCount="272">
   <si>
     <t>#</t>
   </si>
@@ -192,7 +192,7 @@
     <t>R8</t>
   </si>
   <si>
-    <t>R9, R11, R17, R21, R22, R32, R42, R43, R44, R45</t>
+    <t>R9, R11, R17, R21, R22, R32, R34, R35, R36, R42, R43, R44, R45</t>
   </si>
   <si>
     <t>R10</t>
@@ -225,9 +225,6 @@
     <t>R33</t>
   </si>
   <si>
-    <t>R34, R35, R36</t>
-  </si>
-  <si>
     <t>R40</t>
   </si>
   <si>
@@ -270,7 +267,7 @@
     <t>CAP CER 0.1UF 16V X7R 0402</t>
   </si>
   <si>
-    <t>22uF 10V 5Ω ±20% 0805 Tantalum Capacitors ROHS</t>
+    <t>CAP TANT 22UF 20% 10V 0805</t>
   </si>
   <si>
     <t>CAP TANT 10UF 20% 10V 0603</t>
@@ -393,16 +390,13 @@
     <t>RES 470 OHM 1% 1/16W 0402</t>
   </si>
   <si>
-    <t>RES 10K OHM 1% 1/5W 0402</t>
-  </si>
-  <si>
     <t>RES 200K OHM 1% 1/16W 0402</t>
   </si>
   <si>
     <t>50mA 100MΩ 100000 Times 260gf@±50gf 12V Surface Mount SPST SMD Tactile Switches ROHS</t>
   </si>
   <si>
-    <t>SWITCH TACTILE SPST-NO 0.05A 12V</t>
+    <t>None Without bracket 50mA 3.05mm 100000 Times 12V 160gf 2.5mm 1.5mm Round Button Standing paste SPST SMD Tactile Switches ROHS</t>
   </si>
   <si>
     <t>SMD Rotary Encoders ROHS</t>
@@ -492,7 +486,7 @@
     <t>TP12422673</t>
   </si>
   <si>
-    <t>B3U-1000P</t>
+    <t>GT-TC032A-H015-L1</t>
   </si>
   <si>
     <t>EC05E1220401</t>
@@ -525,7 +519,7 @@
     <t>CC0402JRX7R7BB104</t>
   </si>
   <si>
-    <t>TCTP1A226M8R</t>
+    <t>TLJR226M010R3800</t>
   </si>
   <si>
     <t>TR8M106M010C2000</t>
@@ -639,9 +633,6 @@
     <t>RC0402FR-07470RL</t>
   </si>
   <si>
-    <t>SR0402FR-7T10KL</t>
-  </si>
-  <si>
     <t>RC0402FR-07200KL</t>
   </si>
   <si>
@@ -672,7 +663,7 @@
     <t>Yageo</t>
   </si>
   <si>
-    <t>Rohm</t>
+    <t>Kyocera AVX</t>
   </si>
   <si>
     <t>Vishay Sprague</t>
@@ -729,7 +720,7 @@
     <t>ROCPU Switch</t>
   </si>
   <si>
-    <t>Omron</t>
+    <t>G-Switch</t>
   </si>
   <si>
     <t>ALPSALPINE</t>
@@ -819,31 +810,31 @@
     <t>Quantity</t>
   </si>
   <si>
+    <t>value</t>
+  </si>
+  <si>
+    <t>Remarks</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>DO NOT PLACE</t>
+  </si>
+  <si>
+    <t>LCD</t>
+  </si>
+  <si>
+    <t>IPS 1.8 inch 15PIN SPI 262K Color TFT LCD Capacitive Round Screen ST77916 Drive IC 360(RGB)*360 Intelligent Wear Knob Screen</t>
+  </si>
+  <si>
+    <t>Aliexpress</t>
+  </si>
+  <si>
     <t>Battery</t>
   </si>
   <si>
-    <t>LCD</t>
-  </si>
-  <si>
-    <t>IPS 1.8 inch 15PIN SPI 262K Color TFT LCD Capacitive Round Screen ST77916 Drive IC 360(RGB)*360 Intelligent Wear Knob Screen</t>
-  </si>
-  <si>
-    <t>-</t>
-  </si>
-  <si>
-    <t>Aliexpress</t>
-  </si>
-  <si>
     <t>3.7V 2000mAh 103450 Battery Lithium Polymer Batteries for POS Machines Bluetooth Speakers Anti-lost Devices Toys Camping Lights</t>
-  </si>
-  <si>
-    <t>Remarks</t>
-  </si>
-  <si>
-    <t>value</t>
-  </si>
-  <si>
-    <t>DO NOT PLACE</t>
   </si>
 </sst>
 </file>
@@ -894,14 +885,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="10"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <strike/>
       <sz val="9"/>
       <color rgb="FFFF0000"/>
@@ -914,6 +897,14 @@
       <strike/>
       <sz val="10"/>
       <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1033,7 +1024,7 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -1075,16 +1066,16 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="7" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1375,20 +1366,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:K60"/>
+  <dimension ref="A1:K59"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3.140625" style="4" customWidth="1"/>
-    <col min="3" max="3" width="18.7109375" style="4" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.140625" style="4" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="36" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="30" customWidth="1"/>
+    <col min="5" max="5" width="29.85546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="20" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="25.28515625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="21.42578125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="5.85546875" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1416,25 +1406,25 @@
         <v>23</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>273</v>
+        <v>263</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>272</v>
+        <v>264</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1450,19 +1440,19 @@
         <v>24</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="J3" s="7">
         <v>3</v>
@@ -1472,7 +1462,7 @@
     <row r="4" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1"/>
       <c r="B4" s="11">
-        <f t="shared" ref="B4:B60" si="0">ROW(B4) - ROW($B$2)</f>
+        <f t="shared" ref="B4:B56" si="0">ROW(B4) - ROW($B$2)</f>
         <v>2</v>
       </c>
       <c r="C4" s="13" t="s">
@@ -1482,51 +1472,51 @@
         <v>25</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="I4" s="10" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="J4" s="9">
         <v>9</v>
       </c>
       <c r="K4" s="9"/>
     </row>
-    <row r="5" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1"/>
       <c r="B5" s="11">
         <f>ROW(B5) - ROW($B$2)</f>
         <v>3</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D5" s="7" t="s">
         <v>26</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="I5" s="8" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="J5" s="7">
         <v>1</v>
@@ -1546,19 +1536,19 @@
         <v>27</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="G6" s="10" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="I6" s="10" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="J6" s="9">
         <v>1</v>
@@ -1578,19 +1568,19 @@
         <v>28</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="J7" s="7">
         <v>3</v>
@@ -1610,19 +1600,19 @@
         <v>29</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F8" s="9" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="G8" s="10" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="H8" s="9" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="I8" s="10" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="J8" s="9">
         <v>1</v>
@@ -1642,19 +1632,19 @@
         <v>30</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="H9" s="7" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="I9" s="8" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="J9" s="7">
         <v>1</v>
@@ -1674,19 +1664,19 @@
         <v>31</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F10" s="9" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="G10" s="10" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="H10" s="9" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="I10" s="10" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="J10" s="9">
         <v>1</v>
@@ -1706,19 +1696,19 @@
         <v>32</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="I11" s="8" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="J11" s="7">
         <v>1</v>
@@ -1738,19 +1728,19 @@
         <v>33</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="F12" s="9" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="G12" s="10" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="H12" s="9" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="I12" s="10" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="J12" s="9">
         <v>1</v>
@@ -1770,19 +1760,19 @@
         <v>34</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="G13" s="8" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="H13" s="7" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="I13" s="8" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="J13" s="7">
         <v>2</v>
@@ -1802,19 +1792,19 @@
         <v>35</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="F14" s="9" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="G14" s="10" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="H14" s="9" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="I14" s="10" t="s">
-        <v>269</v>
+        <v>265</v>
       </c>
       <c r="J14" s="9">
         <v>4</v>
@@ -1834,19 +1824,19 @@
         <v>36</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="G15" s="8" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="I15" s="10" t="s">
-        <v>269</v>
+        <v>265</v>
       </c>
       <c r="J15" s="7">
         <v>1</v>
@@ -1866,19 +1856,19 @@
         <v>37</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="F16" s="9" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="G16" s="10" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="H16" s="9" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="I16" s="10" t="s">
-        <v>269</v>
+        <v>265</v>
       </c>
       <c r="J16" s="9">
         <v>6</v>
@@ -1898,19 +1888,19 @@
         <v>38</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="G17" s="8" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="H17" s="7" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="I17" s="10" t="s">
-        <v>269</v>
+        <v>265</v>
       </c>
       <c r="J17" s="7">
         <v>1</v>
@@ -1930,19 +1920,19 @@
         <v>39</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F18" s="9" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G18" s="10" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="H18" s="9" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="I18" s="10" t="s">
-        <v>269</v>
+        <v>265</v>
       </c>
       <c r="J18" s="9">
         <v>1</v>
@@ -1962,19 +1952,19 @@
         <v>40</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>269</v>
+        <v>265</v>
       </c>
       <c r="G19" s="8" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="H19" s="7" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="I19" s="10" t="s">
-        <v>269</v>
+        <v>265</v>
       </c>
       <c r="J19" s="7">
         <v>1</v>
@@ -1994,19 +1984,19 @@
         <v>41</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F20" s="7" t="s">
-        <v>269</v>
+        <v>265</v>
       </c>
       <c r="G20" s="10" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="H20" s="9" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="I20" s="10" t="s">
-        <v>269</v>
+        <v>265</v>
       </c>
       <c r="J20" s="9">
         <v>1</v>
@@ -2026,19 +2016,19 @@
         <v>42</v>
       </c>
       <c r="E21" s="8" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="F21" s="7" t="s">
-        <v>269</v>
+        <v>265</v>
       </c>
       <c r="G21" s="8" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="H21" s="7" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="I21" s="10" t="s">
-        <v>269</v>
+        <v>265</v>
       </c>
       <c r="J21" s="7">
         <v>1</v>
@@ -2058,19 +2048,19 @@
         <v>43</v>
       </c>
       <c r="E22" s="10" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="F22" s="7" t="s">
-        <v>269</v>
+        <v>265</v>
       </c>
       <c r="G22" s="10" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="H22" s="9" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="I22" s="10" t="s">
-        <v>269</v>
+        <v>265</v>
       </c>
       <c r="J22" s="9">
         <v>1</v>
@@ -2090,19 +2080,19 @@
         <v>44</v>
       </c>
       <c r="E23" s="8" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F23" s="7" t="s">
-        <v>269</v>
+        <v>265</v>
       </c>
       <c r="G23" s="8" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="H23" s="7" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="I23" s="10" t="s">
-        <v>269</v>
+        <v>265</v>
       </c>
       <c r="J23" s="7">
         <v>1</v>
@@ -2122,19 +2112,19 @@
         <v>45</v>
       </c>
       <c r="E24" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F24" s="7" t="s">
-        <v>269</v>
+        <v>265</v>
       </c>
       <c r="G24" s="10" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="H24" s="9" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="I24" s="10" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="J24" s="9">
         <v>1</v>
@@ -2154,19 +2144,19 @@
         <v>46</v>
       </c>
       <c r="E25" s="8" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F25" s="7" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="G25" s="8" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="H25" s="7" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="I25" s="8" t="s">
-        <v>269</v>
+        <v>265</v>
       </c>
       <c r="J25" s="7">
         <v>1</v>
@@ -2186,19 +2176,19 @@
         <v>47</v>
       </c>
       <c r="E26" s="10" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F26" s="9" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="G26" s="10" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="H26" s="9" t="s">
-        <v>230</v>
-      </c>
-      <c r="I26" s="10" t="s">
-        <v>269</v>
+        <v>227</v>
+      </c>
+      <c r="I26" s="8" t="s">
+        <v>265</v>
       </c>
       <c r="J26" s="9">
         <v>2</v>
@@ -2218,19 +2208,19 @@
         <v>48</v>
       </c>
       <c r="E27" s="8" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="F27" s="7" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="G27" s="8" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="H27" s="7" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="I27" s="8" t="s">
-        <v>269</v>
+        <v>265</v>
       </c>
       <c r="J27" s="7">
         <v>1</v>
@@ -2250,19 +2240,19 @@
         <v>49</v>
       </c>
       <c r="E28" s="10" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F28" s="9" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="G28" s="10" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="H28" s="9" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="I28" s="8" t="s">
-        <v>269</v>
+        <v>265</v>
       </c>
       <c r="J28" s="9">
         <v>3</v>
@@ -2282,19 +2272,19 @@
         <v>50</v>
       </c>
       <c r="E29" s="8" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F29" s="7" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="G29" s="8" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="H29" s="7" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="I29" s="8" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="J29" s="7">
         <v>2</v>
@@ -2314,19 +2304,19 @@
         <v>51</v>
       </c>
       <c r="E30" s="10" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="F30" s="9" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="G30" s="10" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="H30" s="9" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="I30" s="10" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="J30" s="9">
         <v>4</v>
@@ -2346,19 +2336,19 @@
         <v>52</v>
       </c>
       <c r="E31" s="8" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F31" s="7" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="G31" s="8" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="H31" s="7" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="I31" s="8" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="J31" s="7">
         <v>2</v>
@@ -2378,19 +2368,19 @@
         <v>53</v>
       </c>
       <c r="E32" s="10" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="F32" s="9" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="G32" s="10" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="H32" s="9" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="I32" s="10" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="J32" s="9">
         <v>4</v>
@@ -2410,26 +2400,26 @@
         <v>54</v>
       </c>
       <c r="E33" s="8" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F33" s="7" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="G33" s="8" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="H33" s="7" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="I33" s="8" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="J33" s="7">
         <v>1</v>
       </c>
       <c r="K33" s="7"/>
     </row>
-    <row r="34" spans="1:11" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="1"/>
       <c r="B34" s="11">
         <f t="shared" si="0"/>
@@ -2438,29 +2428,29 @@
       <c r="C34" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="D34" s="16" t="s">
+      <c r="D34" s="15" t="s">
         <v>55</v>
       </c>
-      <c r="E34" s="17" t="s">
-        <v>110</v>
-      </c>
-      <c r="F34" s="16" t="s">
-        <v>152</v>
-      </c>
-      <c r="G34" s="17" t="s">
-        <v>192</v>
-      </c>
-      <c r="H34" s="16" t="s">
-        <v>216</v>
-      </c>
-      <c r="I34" s="17" t="s">
-        <v>253</v>
-      </c>
-      <c r="J34" s="16">
+      <c r="E34" s="16" t="s">
+        <v>109</v>
+      </c>
+      <c r="F34" s="15" t="s">
+        <v>150</v>
+      </c>
+      <c r="G34" s="16" t="s">
+        <v>190</v>
+      </c>
+      <c r="H34" s="15" t="s">
+        <v>213</v>
+      </c>
+      <c r="I34" s="16" t="s">
+        <v>250</v>
+      </c>
+      <c r="J34" s="15">
         <v>3</v>
       </c>
-      <c r="K34" s="18" t="s">
-        <v>274</v>
+      <c r="K34" s="17" t="s">
+        <v>266</v>
       </c>
     </row>
     <row r="35" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -2476,26 +2466,26 @@
         <v>56</v>
       </c>
       <c r="E35" s="8" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F35" s="7" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="G35" s="8" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="H35" s="7" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="I35" s="8" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="J35" s="7">
         <v>1</v>
       </c>
       <c r="K35" s="7"/>
     </row>
-    <row r="36" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="1"/>
       <c r="B36" s="11">
         <f t="shared" si="0"/>
@@ -2508,22 +2498,22 @@
         <v>57</v>
       </c>
       <c r="E36" s="10" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F36" s="9" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="G36" s="10" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="H36" s="9" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="I36" s="10" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="J36" s="9">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="K36" s="9"/>
     </row>
@@ -2540,19 +2530,19 @@
         <v>58</v>
       </c>
       <c r="E37" s="8" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="F37" s="7" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="G37" s="8" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="H37" s="7" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="I37" s="8" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="J37" s="7">
         <v>1</v>
@@ -2572,19 +2562,19 @@
         <v>59</v>
       </c>
       <c r="E38" s="10" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F38" s="9" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="G38" s="10" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="H38" s="9" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="I38" s="10" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="J38" s="9">
         <v>1</v>
@@ -2604,19 +2594,19 @@
         <v>60</v>
       </c>
       <c r="E39" s="8" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F39" s="7" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="G39" s="8" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="H39" s="7" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="I39" s="8" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="J39" s="7">
         <v>1</v>
@@ -2636,19 +2626,19 @@
         <v>61</v>
       </c>
       <c r="E40" s="10" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="F40" s="9" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="G40" s="10" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="H40" s="9" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="I40" s="10" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="J40" s="9">
         <v>1</v>
@@ -2668,19 +2658,19 @@
         <v>62</v>
       </c>
       <c r="E41" s="8" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F41" s="7" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="G41" s="8" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="H41" s="7" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="I41" s="8" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="J41" s="7">
         <v>1</v>
@@ -2700,19 +2690,19 @@
         <v>63</v>
       </c>
       <c r="E42" s="10" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F42" s="9" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="G42" s="10" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="H42" s="9" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="I42" s="10" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="J42" s="9">
         <v>3</v>
@@ -2732,19 +2722,19 @@
         <v>64</v>
       </c>
       <c r="E43" s="8" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F43" s="7" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="G43" s="8" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="H43" s="7" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="I43" s="8" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="J43" s="7">
         <v>1</v>
@@ -2764,19 +2754,19 @@
         <v>65</v>
       </c>
       <c r="E44" s="10" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F44" s="9" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="G44" s="10" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="H44" s="9" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="I44" s="10" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="J44" s="9">
         <v>2</v>
@@ -2796,19 +2786,19 @@
         <v>66</v>
       </c>
       <c r="E45" s="8" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F45" s="7" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="G45" s="8" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="H45" s="7" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="I45" s="8" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="J45" s="7">
         <v>2</v>
@@ -2828,19 +2818,19 @@
         <v>67</v>
       </c>
       <c r="E46" s="10" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="F46" s="9" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="G46" s="10" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="H46" s="9" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="I46" s="10" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="J46" s="9">
         <v>1</v>
@@ -2853,29 +2843,29 @@
         <f>ROW(B47) - ROW($B$2)</f>
         <v>45</v>
       </c>
-      <c r="C47" s="13" t="s">
+      <c r="C47" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D47" s="7" t="s">
         <v>68</v>
       </c>
       <c r="E47" s="8" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F47" s="7" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="G47" s="8" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="H47" s="7" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="I47" s="8" t="s">
-        <v>255</v>
+        <v>261</v>
       </c>
       <c r="J47" s="7">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K47" s="7"/>
     </row>
@@ -2886,94 +2876,94 @@
         <v>46</v>
       </c>
       <c r="C48" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="D48" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="D48" s="15" t="s">
         <v>69</v>
       </c>
-      <c r="E48" s="10" t="s">
-        <v>125</v>
-      </c>
-      <c r="F48" s="9" t="s">
-        <v>153</v>
-      </c>
-      <c r="G48" s="10" t="s">
-        <v>207</v>
-      </c>
-      <c r="H48" s="9" t="s">
-        <v>216</v>
-      </c>
-      <c r="I48" s="10" t="s">
-        <v>264</v>
-      </c>
-      <c r="J48" s="9">
-        <v>1</v>
-      </c>
-      <c r="K48" s="9"/>
-    </row>
-    <row r="49" spans="1:11" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E48" s="16" t="s">
+        <v>107</v>
+      </c>
+      <c r="F48" s="15" t="s">
+        <v>151</v>
+      </c>
+      <c r="G48" s="16" t="s">
+        <v>188</v>
+      </c>
+      <c r="H48" s="15" t="s">
+        <v>213</v>
+      </c>
+      <c r="I48" s="16" t="s">
+        <v>250</v>
+      </c>
+      <c r="J48" s="15">
+        <v>1</v>
+      </c>
+      <c r="K48" s="17" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="49" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A49" s="1"/>
       <c r="B49" s="11">
         <f>ROW(B49) - ROW($B$2)</f>
         <v>47</v>
       </c>
       <c r="C49" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="D49" s="16" t="s">
+        <v>18</v>
+      </c>
+      <c r="D49" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="E49" s="17" t="s">
-        <v>108</v>
-      </c>
-      <c r="F49" s="16" t="s">
-        <v>153</v>
-      </c>
-      <c r="G49" s="17" t="s">
-        <v>190</v>
-      </c>
-      <c r="H49" s="16" t="s">
-        <v>216</v>
-      </c>
-      <c r="I49" s="17" t="s">
-        <v>253</v>
-      </c>
-      <c r="J49" s="16">
-        <v>1</v>
-      </c>
-      <c r="K49" s="18" t="s">
-        <v>274</v>
-      </c>
-    </row>
-    <row r="50" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E49" s="8" t="s">
+        <v>124</v>
+      </c>
+      <c r="F49" s="7" t="s">
+        <v>265</v>
+      </c>
+      <c r="G49" s="8" t="s">
+        <v>154</v>
+      </c>
+      <c r="H49" s="7" t="s">
+        <v>232</v>
+      </c>
+      <c r="I49" s="8" t="s">
+        <v>265</v>
+      </c>
+      <c r="J49" s="7">
+        <v>2</v>
+      </c>
+      <c r="K49" s="7"/>
+    </row>
+    <row r="50" spans="1:11" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A50" s="1"/>
       <c r="B50" s="11">
         <f t="shared" si="0"/>
         <v>48</v>
       </c>
       <c r="C50" s="13" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D50" s="9" t="s">
         <v>71</v>
       </c>
       <c r="E50" s="10" t="s">
-        <v>126</v>
-      </c>
-      <c r="F50" s="9" t="s">
-        <v>269</v>
+        <v>125</v>
+      </c>
+      <c r="F50" s="7" t="s">
+        <v>265</v>
       </c>
       <c r="G50" s="10" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="H50" s="9" t="s">
-        <v>235</v>
-      </c>
-      <c r="I50" s="10" t="s">
-        <v>269</v>
+        <v>233</v>
+      </c>
+      <c r="I50" s="8" t="s">
+        <v>265</v>
       </c>
       <c r="J50" s="9">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K50" s="9"/>
     </row>
@@ -2984,57 +2974,57 @@
         <v>49</v>
       </c>
       <c r="C51" s="12" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D51" s="7" t="s">
         <v>72</v>
       </c>
       <c r="E51" s="8" t="s">
-        <v>127</v>
-      </c>
-      <c r="F51" s="9" t="s">
-        <v>269</v>
+        <v>126</v>
+      </c>
+      <c r="F51" s="7" t="s">
+        <v>265</v>
       </c>
       <c r="G51" s="8" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H51" s="7" t="s">
-        <v>236</v>
-      </c>
-      <c r="I51" s="10" t="s">
-        <v>269</v>
+        <v>234</v>
+      </c>
+      <c r="I51" s="8" t="s">
+        <v>265</v>
       </c>
       <c r="J51" s="7">
         <v>1</v>
       </c>
       <c r="K51" s="7"/>
     </row>
-    <row r="52" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A52" s="1"/>
       <c r="B52" s="11">
         <f t="shared" si="0"/>
         <v>50</v>
       </c>
       <c r="C52" s="13" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D52" s="9" t="s">
         <v>73</v>
       </c>
       <c r="E52" s="10" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F52" s="9" t="s">
-        <v>269</v>
+        <v>157</v>
       </c>
       <c r="G52" s="10" t="s">
-        <v>158</v>
+        <v>205</v>
       </c>
       <c r="H52" s="9" t="s">
-        <v>237</v>
-      </c>
-      <c r="I52" s="10" t="s">
-        <v>269</v>
+        <v>235</v>
+      </c>
+      <c r="I52" s="8" t="s">
+        <v>265</v>
       </c>
       <c r="J52" s="9">
         <v>1</v>
@@ -3054,19 +3044,19 @@
         <v>74</v>
       </c>
       <c r="E53" s="8" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="F53" s="7" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="G53" s="8" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="H53" s="7" t="s">
-        <v>238</v>
-      </c>
-      <c r="I53" s="10" t="s">
-        <v>269</v>
+        <v>236</v>
+      </c>
+      <c r="I53" s="8" t="s">
+        <v>265</v>
       </c>
       <c r="J53" s="7">
         <v>1</v>
@@ -3086,26 +3076,26 @@
         <v>75</v>
       </c>
       <c r="E54" s="10" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F54" s="9" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="G54" s="10" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="H54" s="9" t="s">
-        <v>239</v>
-      </c>
-      <c r="I54" s="10" t="s">
-        <v>269</v>
+        <v>237</v>
+      </c>
+      <c r="I54" s="8" t="s">
+        <v>265</v>
       </c>
       <c r="J54" s="9">
         <v>1</v>
       </c>
       <c r="K54" s="9"/>
     </row>
-    <row r="55" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A55" s="1"/>
       <c r="B55" s="11">
         <f>ROW(B55) - ROW($B$2)</f>
@@ -3118,26 +3108,26 @@
         <v>76</v>
       </c>
       <c r="E55" s="8" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F55" s="7" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="G55" s="8" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="H55" s="7" t="s">
-        <v>240</v>
-      </c>
-      <c r="I55" s="10" t="s">
-        <v>269</v>
+        <v>237</v>
+      </c>
+      <c r="I55" s="8" t="s">
+        <v>265</v>
       </c>
       <c r="J55" s="7">
         <v>1</v>
       </c>
       <c r="K55" s="7"/>
     </row>
-    <row r="56" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A56" s="1"/>
       <c r="B56" s="11">
         <f t="shared" si="0"/>
@@ -3150,153 +3140,121 @@
         <v>77</v>
       </c>
       <c r="E56" s="10" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F56" s="9" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="G56" s="10" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="H56" s="9" t="s">
-        <v>240</v>
-      </c>
-      <c r="I56" s="10" t="s">
-        <v>269</v>
+        <v>219</v>
+      </c>
+      <c r="I56" s="8" t="s">
+        <v>265</v>
       </c>
       <c r="J56" s="9">
         <v>1</v>
       </c>
       <c r="K56" s="9"/>
     </row>
-    <row r="57" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A57" s="1"/>
       <c r="B57" s="11">
         <f>ROW(B57) - ROW($B$2)</f>
         <v>55</v>
       </c>
       <c r="C57" s="12" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D57" s="7" t="s">
         <v>78</v>
       </c>
       <c r="E57" s="8" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="F57" s="7" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="G57" s="8" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="H57" s="7" t="s">
-        <v>222</v>
-      </c>
-      <c r="I57" s="10" t="s">
+        <v>238</v>
+      </c>
+      <c r="I57" s="8" t="s">
+        <v>265</v>
+      </c>
+      <c r="J57" s="7">
+        <v>1</v>
+      </c>
+      <c r="K57" s="7"/>
+    </row>
+    <row r="58" spans="1:11" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B58" s="11">
+        <f t="shared" ref="B58:B59" si="1">ROW(B58) - ROW($B$2)</f>
+        <v>56</v>
+      </c>
+      <c r="C58" s="13" t="s">
+        <v>267</v>
+      </c>
+      <c r="D58" s="9" t="s">
+        <v>265</v>
+      </c>
+      <c r="E58" s="10" t="s">
+        <v>268</v>
+      </c>
+      <c r="F58" s="9" t="s">
+        <v>265</v>
+      </c>
+      <c r="G58" s="10" t="s">
+        <v>267</v>
+      </c>
+      <c r="H58" s="9" t="s">
+        <v>265</v>
+      </c>
+      <c r="I58" s="10" t="s">
+        <v>265</v>
+      </c>
+      <c r="J58" s="9">
+        <v>1</v>
+      </c>
+      <c r="K58" s="18" t="s">
         <v>269</v>
       </c>
-      <c r="J57" s="7">
-        <v>1</v>
-      </c>
-      <c r="K57" s="7"/>
-    </row>
-    <row r="58" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A58" s="1"/>
-      <c r="B58" s="11">
-        <f t="shared" si="0"/>
-        <v>56</v>
-      </c>
-      <c r="C58" s="13" t="s">
-        <v>22</v>
-      </c>
-      <c r="D58" s="9" t="s">
-        <v>79</v>
-      </c>
-      <c r="E58" s="10" t="s">
-        <v>134</v>
-      </c>
-      <c r="F58" s="9" t="s">
-        <v>164</v>
-      </c>
-      <c r="G58" s="10" t="s">
-        <v>213</v>
-      </c>
-      <c r="H58" s="9" t="s">
-        <v>241</v>
-      </c>
-      <c r="I58" s="10" t="s">
-        <v>269</v>
-      </c>
-      <c r="J58" s="9">
-        <v>1</v>
-      </c>
-      <c r="K58" s="9"/>
     </row>
     <row r="59" spans="1:11" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B59" s="11">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>57</v>
       </c>
       <c r="C59" s="13" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="D59" s="9" t="s">
-        <v>269</v>
+        <v>265</v>
       </c>
       <c r="E59" s="10" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="F59" s="9" t="s">
-        <v>269</v>
+        <v>265</v>
       </c>
       <c r="G59" s="10" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="H59" s="9" t="s">
-        <v>269</v>
+        <v>265</v>
       </c>
       <c r="I59" s="10" t="s">
-        <v>269</v>
+        <v>265</v>
       </c>
       <c r="J59" s="9">
         <v>1</v>
       </c>
-      <c r="K59" s="15" t="s">
+      <c r="K59" s="18" t="s">
         <v>270</v>
-      </c>
-    </row>
-    <row r="60" spans="1:11" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B60" s="11">
-        <f t="shared" si="0"/>
-        <v>58</v>
-      </c>
-      <c r="C60" s="13" t="s">
-        <v>266</v>
-      </c>
-      <c r="D60" s="9" t="s">
-        <v>269</v>
-      </c>
-      <c r="E60" s="10" t="s">
-        <v>271</v>
-      </c>
-      <c r="F60" s="9" t="s">
-        <v>269</v>
-      </c>
-      <c r="G60" s="10" t="s">
-        <v>266</v>
-      </c>
-      <c r="H60" s="9" t="s">
-        <v>269</v>
-      </c>
-      <c r="I60" s="10" t="s">
-        <v>269</v>
-      </c>
-      <c r="J60" s="9">
-        <v>1</v>
-      </c>
-      <c r="K60" s="15" t="s">
-        <v>266</v>
       </c>
     </row>
   </sheetData>
@@ -3304,8 +3262,8 @@
     <mergeCell ref="I1:K1"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="K59" r:id="rId1" location="nav-specification"/>
-    <hyperlink ref="K60" r:id="rId2"/>
+    <hyperlink ref="K58" r:id="rId1" location="nav-specification"/>
+    <hyperlink ref="K59" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId3"/>

</xml_diff>